<commit_message>
Updated toxicity plots for publication
</commit_message>
<xml_diff>
--- a/Zinc/5. Cluster analysis/Clustering by sample results/Relative_freq_percentages_by_cluster.xlsx
+++ b/Zinc/5. Cluster analysis/Clustering by sample results/Relative_freq_percentages_by_cluster.xlsx
@@ -1,92 +1,82 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://irtacat-my.sharepoint.com/personal/cecilia_albert_irta_cat/Documents/Escriptori/Trace-element-bioavailability-spatial-assessment/Zinc/5. Cluster analysis/Clustering by sample results/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_C2CE303C0089EEA2EC45B3CE6F4DDD168C55A94A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C8BE2B95-2FF7-42DF-B9D6-BDD22B221B6B}"/>
+  <workbookPr date1904="false"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet 1'!$A$1:$E$1</definedName>
-  </definedNames>
-  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="19">
-  <si>
-    <t>Variable</t>
-  </si>
-  <si>
-    <t>cluster4</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Freq</t>
-  </si>
-  <si>
-    <t>RelFreq</t>
-  </si>
-  <si>
-    <t>Development</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>High</t>
-  </si>
-  <si>
-    <t>Low</t>
-  </si>
-  <si>
-    <t>Medium</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>Regime</t>
-  </si>
-  <si>
-    <t>NonPerennial</t>
-  </si>
-  <si>
-    <t>Perennial</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>Tributaries</t>
-  </si>
-  <si>
-    <t>Main Stem</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+  <si>
+    <t xml:space="preserve">Variable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cluster4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Freq</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RelFreq</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Development</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regime</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NonPerennial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perennial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tributaries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Main Stem</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -122,15 +112,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -412,14 +393,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E25"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="15.7265625" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -436,7 +414,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -446,14 +424,14 @@
       <c r="C2" t="s">
         <v>7</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="n">
         <v>69</v>
       </c>
-      <c r="E2">
-        <v>56.557377049180303</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E2" t="n">
+        <v>56.5573770491803</v>
+      </c>
+    </row>
+    <row r="3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -463,14 +441,14 @@
       <c r="C3" t="s">
         <v>8</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="n">
         <v>20</v>
       </c>
-      <c r="E3">
-        <v>16.393442622950801</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E3" t="n">
+        <v>16.3934426229508</v>
+      </c>
+    </row>
+    <row r="4">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -480,14 +458,14 @@
       <c r="C4" t="s">
         <v>9</v>
       </c>
-      <c r="D4">
+      <c r="D4" t="n">
         <v>33</v>
       </c>
-      <c r="E4">
+      <c r="E4" t="n">
         <v>27.0491803278689</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -497,14 +475,14 @@
       <c r="C5" t="s">
         <v>8</v>
       </c>
-      <c r="D5">
-        <v>5</v>
-      </c>
-      <c r="E5">
-        <v>35.714285714285701</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D5" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" t="n">
+        <v>35.7142857142857</v>
+      </c>
+    </row>
+    <row r="6">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -514,14 +492,14 @@
       <c r="C6" t="s">
         <v>9</v>
       </c>
-      <c r="D6">
+      <c r="D6" t="n">
         <v>9</v>
       </c>
-      <c r="E6">
-        <v>64.285714285714306</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E6" t="n">
+        <v>64.2857142857143</v>
+      </c>
+    </row>
+    <row r="7">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -531,14 +509,14 @@
       <c r="C7" t="s">
         <v>7</v>
       </c>
-      <c r="D7">
+      <c r="D7" t="n">
         <v>40</v>
       </c>
-      <c r="E7">
-        <v>31.496062992125999</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E7" t="n">
+        <v>31.496062992126</v>
+      </c>
+    </row>
+    <row r="8">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -548,14 +526,14 @@
       <c r="C8" t="s">
         <v>8</v>
       </c>
-      <c r="D8">
+      <c r="D8" t="n">
         <v>29</v>
       </c>
-      <c r="E8">
-        <v>22.834645669291302</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E8" t="n">
+        <v>22.8346456692913</v>
+      </c>
+    </row>
+    <row r="9">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -565,14 +543,14 @@
       <c r="C9" t="s">
         <v>9</v>
       </c>
-      <c r="D9">
+      <c r="D9" t="n">
         <v>58</v>
       </c>
-      <c r="E9">
-        <v>45.669291338582703</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E9" t="n">
+        <v>45.6692913385827</v>
+      </c>
+    </row>
+    <row r="10">
       <c r="A10" t="s">
         <v>5</v>
       </c>
@@ -582,14 +560,14 @@
       <c r="C10" t="s">
         <v>7</v>
       </c>
-      <c r="D10">
+      <c r="D10" t="n">
         <v>10</v>
       </c>
-      <c r="E10">
-        <v>10.752688172042999</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E10" t="n">
+        <v>10.752688172043</v>
+      </c>
+    </row>
+    <row r="11">
       <c r="A11" t="s">
         <v>5</v>
       </c>
@@ -599,14 +577,14 @@
       <c r="C11" t="s">
         <v>8</v>
       </c>
-      <c r="D11">
+      <c r="D11" t="n">
         <v>54</v>
       </c>
-      <c r="E11">
-        <v>58.064516129032299</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E11" t="n">
+        <v>58.0645161290323</v>
+      </c>
+    </row>
+    <row r="12">
       <c r="A12" t="s">
         <v>5</v>
       </c>
@@ -616,14 +594,14 @@
       <c r="C12" t="s">
         <v>9</v>
       </c>
-      <c r="D12">
+      <c r="D12" t="n">
         <v>29</v>
       </c>
-      <c r="E12">
+      <c r="E12" t="n">
         <v>31.1827956989247</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -633,14 +611,14 @@
       <c r="C13" t="s">
         <v>14</v>
       </c>
-      <c r="D13">
-        <v>5</v>
-      </c>
-      <c r="E13">
-        <v>4.0983606557377001</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D13" t="n">
+        <v>5</v>
+      </c>
+      <c r="E13" t="n">
+        <v>4.0983606557377</v>
+      </c>
+    </row>
+    <row r="14">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -650,14 +628,14 @@
       <c r="C14" t="s">
         <v>15</v>
       </c>
-      <c r="D14">
+      <c r="D14" t="n">
         <v>117</v>
       </c>
-      <c r="E14">
-        <v>95.901639344262307</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E14" t="n">
+        <v>95.9016393442623</v>
+      </c>
+    </row>
+    <row r="15">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -667,14 +645,14 @@
       <c r="C15" t="s">
         <v>14</v>
       </c>
-      <c r="D15">
+      <c r="D15" t="n">
         <v>13</v>
       </c>
-      <c r="E15">
-        <v>92.857142857142904</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E15" t="n">
+        <v>92.8571428571429</v>
+      </c>
+    </row>
+    <row r="16">
       <c r="A16" t="s">
         <v>13</v>
       </c>
@@ -684,14 +662,14 @@
       <c r="C16" t="s">
         <v>15</v>
       </c>
-      <c r="D16">
+      <c r="D16" t="n">
         <v>1</v>
       </c>
-      <c r="E16">
-        <v>7.1428571428571397</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E16" t="n">
+        <v>7.14285714285714</v>
+      </c>
+    </row>
+    <row r="17">
       <c r="A17" t="s">
         <v>13</v>
       </c>
@@ -701,14 +679,14 @@
       <c r="C17" t="s">
         <v>15</v>
       </c>
-      <c r="D17">
+      <c r="D17" t="n">
         <v>127</v>
       </c>
-      <c r="E17">
+      <c r="E17" t="n">
         <v>100</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18">
       <c r="A18" t="s">
         <v>13</v>
       </c>
@@ -718,14 +696,14 @@
       <c r="C18" t="s">
         <v>14</v>
       </c>
-      <c r="D18">
+      <c r="D18" t="n">
         <v>29</v>
       </c>
-      <c r="E18">
+      <c r="E18" t="n">
         <v>31.1827956989247</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19">
       <c r="A19" t="s">
         <v>13</v>
       </c>
@@ -735,14 +713,14 @@
       <c r="C19" t="s">
         <v>15</v>
       </c>
-      <c r="D19">
+      <c r="D19" t="n">
         <v>64</v>
       </c>
-      <c r="E19">
-        <v>68.817204301075293</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E19" t="n">
+        <v>68.8172043010753</v>
+      </c>
+    </row>
+    <row r="20">
       <c r="A20" t="s">
         <v>16</v>
       </c>
@@ -752,14 +730,14 @@
       <c r="C20" t="s">
         <v>17</v>
       </c>
-      <c r="D20">
+      <c r="D20" t="n">
         <v>122</v>
       </c>
-      <c r="E20">
+      <c r="E20" t="n">
         <v>100</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21">
       <c r="A21" t="s">
         <v>16</v>
       </c>
@@ -769,14 +747,14 @@
       <c r="C21" t="s">
         <v>17</v>
       </c>
-      <c r="D21">
+      <c r="D21" t="n">
         <v>14</v>
       </c>
-      <c r="E21">
+      <c r="E21" t="n">
         <v>100</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22">
       <c r="A22" t="s">
         <v>16</v>
       </c>
@@ -786,14 +764,14 @@
       <c r="C22" t="s">
         <v>18</v>
       </c>
-      <c r="D22">
+      <c r="D22" t="n">
         <v>97</v>
       </c>
-      <c r="E22">
-        <v>76.377952755905497</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="E22" t="n">
+        <v>76.3779527559055</v>
+      </c>
+    </row>
+    <row r="23">
       <c r="A23" t="s">
         <v>16</v>
       </c>
@@ -803,14 +781,14 @@
       <c r="C23" t="s">
         <v>17</v>
       </c>
-      <c r="D23">
+      <c r="D23" t="n">
         <v>30</v>
       </c>
-      <c r="E23">
+      <c r="E23" t="n">
         <v>23.6220472440945</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24">
       <c r="A24" t="s">
         <v>16</v>
       </c>
@@ -820,14 +798,14 @@
       <c r="C24" t="s">
         <v>18</v>
       </c>
-      <c r="D24">
+      <c r="D24" t="n">
         <v>9</v>
       </c>
-      <c r="E24">
+      <c r="E24" t="n">
         <v>9.67741935483871</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25">
       <c r="A25" t="s">
         <v>16</v>
       </c>
@@ -837,16 +815,15 @@
       <c r="C25" t="s">
         <v>17</v>
       </c>
-      <c r="D25">
+      <c r="D25" t="n">
         <v>84</v>
       </c>
-      <c r="E25">
-        <v>90.322580645161295</v>
+      <c r="E25" t="n">
+        <v>90.3225806451613</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated publication plots - renamed cluster 2 to 3 and 3 to 2
</commit_message>
<xml_diff>
--- a/Zinc/5. Cluster analysis/Clustering by sample results/Relative_freq_percentages_by_cluster.xlsx
+++ b/Zinc/5. Cluster analysis/Clustering by sample results/Relative_freq_percentages_by_cluster.xlsx
@@ -44,10 +44,10 @@
     <t xml:space="preserve">Medium</t>
   </si>
   <si>
+    <t xml:space="preserve">3</t>
+  </si>
+  <si>
     <t xml:space="preserve">2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3</t>
   </si>
   <si>
     <t xml:space="preserve">4</t>

</xml_diff>